<commit_message>
fix: update reviewer titles to neutral roles and refine evaluation wording
</commit_message>
<xml_diff>
--- a/data/netsage_summary_metrics.xlsx
+++ b/data/netsage_summary_metrics.xlsx
@@ -834,17 +834,17 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tested in component suite</t>
+          <t>AI diagnosis correctly identified Fa0/2 assigned to VLAN 20 instead of 10 based on show vlan brief.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Test Reviewer</t>
+          <t>Human Reviewer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-09-30 17:38:56</t>
+          <t>2026-09-30 18:20:39</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Alice Chen (Student)</t>
+          <t>Student Reviewer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Alice Chen (Student)</t>
+          <t>Student Reviewer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bob Patel (Student)</t>
+          <t>Project Team</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Prof. Miller (CCNP)</t>
+          <t>Human Reviewer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Bob Patel (Student)</t>
+          <t>Project Team</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Alice Chen (Student)</t>
+          <t>Student Reviewer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bob Patel (Student)</t>
+          <t>Project Team</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Prof. Miller (CCNP)</t>
+          <t>Human Reviewer</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Prof. Miller (CCNP)</t>
+          <t>Human Reviewer</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Prof. Miller (CCNP)</t>
+          <t>Human Reviewer</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Prof. Miller (CCNP)</t>
+          <t>Human Reviewer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">

</xml_diff>